<commit_message>
ui updates with results
</commit_message>
<xml_diff>
--- a/HSLedger_Trading_Module/output/HSLedger_Equity_CGT_Report.xlsx
+++ b/HSLedger_Trading_Module/output/HSLedger_Equity_CGT_Report.xlsx
@@ -593,7 +593,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 27/04/2026</t>
+          <t>Generated: 28/04/2026</t>
         </is>
       </c>
     </row>
@@ -18300,7 +18300,7 @@
         <v>45614</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="H2" s="7" t="b">
         <v>1</v>
@@ -18333,7 +18333,7 @@
         <v>45719</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H3" s="9" t="b">
         <v>1</v>
@@ -18366,7 +18366,7 @@
         <v>45744</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="H4" s="7" t="b">
         <v>1</v>
@@ -18399,7 +18399,7 @@
         <v>45772</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="H5" s="9" t="b">
         <v>1</v>
@@ -18432,7 +18432,7 @@
         <v>45610</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="H6" s="7" t="b">
         <v>1</v>
@@ -18465,7 +18465,7 @@
         <v>45663</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="H7" s="9" t="b">
         <v>1</v>
@@ -18498,7 +18498,7 @@
         <v>45672</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="H8" s="7" t="b">
         <v>1</v>
@@ -18531,7 +18531,7 @@
         <v>45708</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H9" s="9" t="b">
         <v>1</v>
@@ -18564,7 +18564,7 @@
         <v>45770</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="H10" s="7" t="b">
         <v>1</v>
@@ -18597,7 +18597,7 @@
         <v>45784</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="H11" s="9" t="b">
         <v>0</v>
@@ -18630,7 +18630,7 @@
         <v>45789</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="H12" s="7" t="b">
         <v>0</v>
@@ -18663,7 +18663,7 @@
         <v>45595</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="H13" s="9" t="b">
         <v>1</v>
@@ -18696,7 +18696,7 @@
         <v>45602</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="H14" s="7" t="b">
         <v>1</v>
@@ -18729,7 +18729,7 @@
         <v>45733</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="H15" s="9" t="b">
         <v>1</v>
@@ -18762,7 +18762,7 @@
         <v>45750</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="H16" s="7" t="b">
         <v>1</v>
@@ -18795,7 +18795,7 @@
         <v>45775</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H17" s="9" t="b">
         <v>1</v>
@@ -18828,7 +18828,7 @@
         <v>45786</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="H18" s="7" t="b">
         <v>0</v>
@@ -18861,7 +18861,7 @@
         <v>45698</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="H19" s="9" t="b">
         <v>1</v>
@@ -18894,7 +18894,7 @@
         <v>45763</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="H20" s="7" t="b">
         <v>1</v>
@@ -18927,7 +18927,7 @@
         <v>45597</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="H21" s="9" t="b">
         <v>1</v>
@@ -18960,7 +18960,7 @@
         <v>45603</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="H22" s="7" t="b">
         <v>1</v>
@@ -18993,7 +18993,7 @@
         <v>45616</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="H23" s="9" t="b">
         <v>1</v>
@@ -19026,7 +19026,7 @@
         <v>45624</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="H24" s="7" t="b">
         <v>1</v>
@@ -19059,7 +19059,7 @@
         <v>45652</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="H25" s="9" t="b">
         <v>1</v>
@@ -19092,7 +19092,7 @@
         <v>45679</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="H26" s="7" t="b">
         <v>1</v>
@@ -19125,7 +19125,7 @@
         <v>45681</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="H27" s="9" t="b">
         <v>1</v>
@@ -19158,7 +19158,7 @@
         <v>45777</v>
       </c>
       <c r="G28" s="7" t="n">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H28" s="7" t="b">
         <v>0</v>
@@ -19191,7 +19191,7 @@
         <v>45793</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="H29" s="9" t="b">
         <v>0</v>
@@ -19224,7 +19224,7 @@
         <v>45504</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="H30" s="7" t="b">
         <v>1</v>
@@ -19257,7 +19257,7 @@
         <v>45611</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="H31" s="9" t="b">
         <v>1</v>
@@ -19290,7 +19290,7 @@
         <v>45651</v>
       </c>
       <c r="G32" s="7" t="n">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="H32" s="7" t="b">
         <v>1</v>
@@ -19323,7 +19323,7 @@
         <v>45749</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="H33" s="9" t="b">
         <v>1</v>
@@ -19356,7 +19356,7 @@
         <v>45777</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H34" s="7" t="b">
         <v>0</v>
@@ -19389,7 +19389,7 @@
         <v>45806</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="H35" s="9" t="b">
         <v>0</v>
@@ -19422,7 +19422,7 @@
         <v>45733</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="H36" s="7" t="b">
         <v>1</v>
@@ -19455,7 +19455,7 @@
         <v>45737</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="H37" s="9" t="b">
         <v>1</v>
@@ -19488,7 +19488,7 @@
         <v>45768</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="H38" s="7" t="b">
         <v>1</v>
@@ -19521,7 +19521,7 @@
         <v>45688</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="H39" s="9" t="b">
         <v>1</v>
@@ -19554,7 +19554,7 @@
         <v>45700</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="H40" s="7" t="b">
         <v>1</v>
@@ -19587,7 +19587,7 @@
         <v>45715</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="H41" s="9" t="b">
         <v>1</v>
@@ -19620,7 +19620,7 @@
         <v>45750</v>
       </c>
       <c r="G42" s="7" t="n">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="H42" s="7" t="b">
         <v>1</v>
@@ -19653,7 +19653,7 @@
         <v>45771</v>
       </c>
       <c r="G43" s="9" t="n">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="H43" s="9" t="b">
         <v>1</v>
@@ -19686,7 +19686,7 @@
         <v>45771</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="H44" s="7" t="b">
         <v>1</v>
@@ -19719,7 +19719,7 @@
         <v>45775</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="H45" s="9" t="b">
         <v>1</v>
@@ -19752,7 +19752,7 @@
         <v>45782</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="H46" s="7" t="b">
         <v>0</v>
@@ -19785,7 +19785,7 @@
         <v>45803</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="H47" s="9" t="b">
         <v>0</v>
@@ -19818,7 +19818,7 @@
         <v>45805</v>
       </c>
       <c r="G48" s="7" t="n">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="H48" s="7" t="b">
         <v>0</v>
@@ -19851,7 +19851,7 @@
         <v>45798</v>
       </c>
       <c r="G49" s="9" t="n">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H49" s="9" t="b">
         <v>0</v>

</xml_diff>